<commit_message>
Add comprehensive data type verification tests and regenerate sample outputs
- Add verification tests using actual EXCEL_FORMATS constants for Currency,
  Integer, Decimal, and Text (matching existing Date test pattern)
- Add test for currency values with symbols using actual EXCEL_FORMATS
- Add end-to-end customized output test for currency value and format
- Regenerate all sample_data/sample_output files with current code to
  reflect proper type coercion (dates as datetime, numbers as numeric)

Agent-Logs-Url: https://github.com/Torbeck/HTR_RaceCharts_Converter/sessions/6043e0ac-2976-4907-ba65-37d7afa22d10

Co-authored-by: ktorbeck <6749800+ktorbeck@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sample_data/sample_output/AQU0322F.xlsx
+++ b/sample_data/sample_output/AQU0322F.xlsx
@@ -18,9 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -61,10 +62,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -717,7 +718,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -2190,10 +2191,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B2" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>1</v>
@@ -2562,10 +2561,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B3" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>1</v>
@@ -3054,10 +3051,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B4" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>1</v>
@@ -3540,10 +3535,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B5" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>1</v>
@@ -4032,10 +4025,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B6" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>1</v>
@@ -4522,10 +4513,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B7" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>1</v>
@@ -5004,10 +4993,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B8" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>2</v>
@@ -5402,10 +5389,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B9" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>2</v>
@@ -5916,10 +5901,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B10" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>2</v>
@@ -6438,10 +6421,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B11" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>2</v>
@@ -6954,10 +6935,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B12" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>2</v>
@@ -7464,10 +7443,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B13" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C13" s="4" t="n">
         <v>2</v>
@@ -7982,10 +7959,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B14" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C14" s="4" t="n">
         <v>3</v>
@@ -8506,10 +8481,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B15" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C15" s="4" t="n">
         <v>3</v>
@@ -9036,10 +9009,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B16" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C16" s="4" t="n">
         <v>3</v>
@@ -9558,10 +9529,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B17" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C17" s="4" t="n">
         <v>3</v>
@@ -10074,10 +10043,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B18" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>3</v>
@@ -10586,10 +10553,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B19" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C19" s="4" t="n">
         <v>3</v>
@@ -11106,10 +11071,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B20" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>4</v>
@@ -11638,10 +11601,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B21" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>4</v>
@@ -12164,10 +12125,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B22" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C22" s="4" t="n">
         <v>4</v>
@@ -12694,10 +12653,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B23" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C23" s="4" t="n">
         <v>4</v>
@@ -13218,10 +13175,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B24" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C24" s="4" t="n">
         <v>4</v>
@@ -13746,10 +13701,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B25" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C25" s="4" t="n">
         <v>4</v>
@@ -14254,10 +14207,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B26" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C26" s="4" t="n">
         <v>5</v>
@@ -14692,10 +14643,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B27" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C27" s="4" t="n">
         <v>5</v>
@@ -15244,10 +15193,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B28" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C28" s="4" t="n">
         <v>5</v>
@@ -15798,10 +15745,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B29" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C29" s="4" t="n">
         <v>5</v>
@@ -16378,10 +16323,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B30" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C30" s="4" t="n">
         <v>5</v>
@@ -16926,10 +16869,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B31" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C31" s="4" t="n">
         <v>5</v>
@@ -17474,10 +17415,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B32" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C32" s="4" t="n">
         <v>5</v>
@@ -18038,10 +17977,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B33" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C33" s="4" t="n">
         <v>6</v>
@@ -18440,10 +18377,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B34" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C34" s="4" t="n">
         <v>6</v>
@@ -18960,10 +18895,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B35" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C35" s="4" t="n">
         <v>6</v>
@@ -19482,10 +19415,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B36" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C36" s="4" t="n">
         <v>6</v>
@@ -19994,10 +19925,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B37" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C37" s="4" t="n">
         <v>6</v>
@@ -20508,10 +20437,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B38" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C38" s="4" t="n">
         <v>6</v>
@@ -21022,10 +20949,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B39" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C39" s="4" t="n">
         <v>7</v>
@@ -21586,10 +21511,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B40" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C40" s="4" t="n">
         <v>7</v>
@@ -22124,10 +22047,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B41" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C41" s="4" t="n">
         <v>7</v>
@@ -22660,10 +22581,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B42" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C42" s="4" t="n">
         <v>7</v>
@@ -23194,10 +23113,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B43" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C43" s="4" t="n">
         <v>7</v>
@@ -23724,10 +23641,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B44" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C44" s="4" t="n">
         <v>7</v>
@@ -24254,10 +24169,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B45" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C45" s="4" t="n">
         <v>7</v>
@@ -24790,10 +24703,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B46" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C46" s="4" t="n">
         <v>7</v>
@@ -25326,10 +25237,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B47" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C47" s="4" t="n">
         <v>8</v>
@@ -25790,10 +25699,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B48" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C48" s="4" t="n">
         <v>8</v>
@@ -26392,10 +26299,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B49" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C49" s="4" t="n">
         <v>8</v>
@@ -26974,10 +26879,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B50" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C50" s="4" t="n">
         <v>8</v>
@@ -27556,10 +27459,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B51" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C51" s="4" t="n">
         <v>8</v>
@@ -28162,10 +28063,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B52" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C52" s="4" t="n">
         <v>8</v>
@@ -28744,10 +28643,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B53" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C53" s="4" t="n">
         <v>8</v>
@@ -29322,10 +29219,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B54" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C54" s="4" t="n">
         <v>8</v>
@@ -29898,10 +29793,8 @@
           <t>AQU</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>03/22/2026</t>
-        </is>
+      <c r="B55" s="3" t="n">
+        <v>46103</v>
       </c>
       <c r="C55" s="4" t="n">
         <v>8</v>

</xml_diff>